<commit_message>
Hotfix: Agregar log de error en Firebase Auth para depurar el inicio de sesion
</commit_message>
<xml_diff>
--- a/Jerarquias por niveles.xlsx
+++ b/Jerarquias por niveles.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giancarlo.lam\Downloads\Planes FERCO V3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE15C546-F409-42F4-A3E8-C2F47651C30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF15888-3C29-40A4-BE90-12035F381EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-2100" windowWidth="19420" windowHeight="10420" xr2:uid="{A3AE2F31-2BAE-421C-A801-465E2044584E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{A3AE2F31-2BAE-421C-A801-465E2044584E}"/>
   </bookViews>
   <sheets>
     <sheet name="Jerarquia" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Jerarquia!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Jerarquia!$A$1:$I$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,31 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="112">
-  <si>
-    <t>Nivel 1</t>
-  </si>
-  <si>
-    <t>Nivel 2</t>
-  </si>
-  <si>
-    <t>Nivel 3</t>
-  </si>
-  <si>
-    <t>Nivel 4</t>
-  </si>
-  <si>
-    <t>Nivel 5</t>
-  </si>
-  <si>
-    <t>Nivel 6</t>
-  </si>
-  <si>
-    <t>Nivel 7</t>
-  </si>
-  <si>
-    <t>Nivel 8</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="106">
   <si>
     <t>Director Comercial GT</t>
   </si>
@@ -336,9 +312,6 @@
     <t>IT</t>
   </si>
   <si>
-    <t>Nivel 9</t>
-  </si>
-  <si>
     <t>Guatemala</t>
   </si>
   <si>
@@ -379,6 +352,15 @@
   </si>
   <si>
     <t>Gerente de Sucursal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">País </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area </t>
+  </si>
+  <si>
+    <t>Puesto</t>
   </si>
 </sst>
 </file>
@@ -794,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B1F15B2-B429-43C8-9EFE-6E439C2435D2}">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -810,49 +792,49 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>104</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>105</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>105</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>105</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -860,268 +842,276 @@
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>80</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G5" s="1"/>
+        <v>102</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>105</v>
+        <v>80</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="1"/>
+        <v>102</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="H9" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="H10" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>8</v>
+      <c r="B13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
@@ -1129,42 +1119,40 @@
     </row>
     <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -1173,19 +1161,19 @@
     </row>
     <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -1194,19 +1182,19 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -1215,63 +1203,63 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="1"/>
+        <v>102</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -1280,144 +1268,144 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
+      <c r="I21" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>26</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>26</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
@@ -1426,19 +1414,19 @@
     </row>
     <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -1447,20 +1435,18 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>36</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -1468,18 +1454,20 @@
     </row>
     <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E29" s="1"/>
+        <v>30</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
@@ -1487,19 +1475,19 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
@@ -1508,20 +1496,18 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
@@ -1529,18 +1515,20 @@
     </row>
     <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E32" s="1"/>
+        <v>36</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
@@ -1548,19 +1536,19 @@
     </row>
     <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -1569,43 +1557,45 @@
     </row>
     <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="E35" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
@@ -1613,22 +1603,22 @@
     </row>
     <row r="36" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
@@ -1636,22 +1626,22 @@
     </row>
     <row r="37" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
@@ -1659,42 +1649,40 @@
     </row>
     <row r="38" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>59</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C39" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
@@ -1703,63 +1691,63 @@
     </row>
     <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F40" s="1"/>
+        <v>56</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
@@ -1768,64 +1756,62 @@
     </row>
     <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F43" s="1"/>
+        <v>63</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>72</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>73</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
@@ -1833,18 +1819,20 @@
     </row>
     <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E46" s="1"/>
+        <v>68</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
@@ -1852,19 +1840,19 @@
     </row>
     <row r="47" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
@@ -1873,43 +1861,45 @@
     </row>
     <row r="48" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F48" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C49" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F49" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
@@ -1917,45 +1907,22 @@
     </row>
     <row r="50" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>86</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
-    </row>
-    <row r="51" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Migracion Fase 1: Inyectar SDK de Supabase y eliminar Firebase de index.html
</commit_message>
<xml_diff>
--- a/Jerarquias por niveles.xlsx
+++ b/Jerarquias por niveles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giancarlo.lam\Downloads\Planes FERCO V3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF15888-3C29-40A4-BE90-12035F381EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43AC953E-CC5F-4079-9C3E-64D83D64F6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{A3AE2F31-2BAE-421C-A801-465E2044584E}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Jerarquia!$A$1:$I$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Jerarquia!$A$1:$J$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="108">
   <si>
     <t>Director Comercial GT</t>
   </si>
@@ -361,6 +361,12 @@
   </si>
   <si>
     <t>Puesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puesto </t>
+  </si>
+  <si>
+    <t>CEO</t>
   </si>
 </sst>
 </file>
@@ -776,21 +782,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B1F15B2-B429-43C8-9EFE-6E439C2435D2}">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="173.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="121.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="112.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" customWidth="1"/>
+    <col min="4" max="4" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="173.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="121.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="112.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>103</v>
       </c>
@@ -798,7 +805,7 @@
         <v>104</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>105</v>
@@ -818,8 +825,11 @@
       <c r="I1" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>89</v>
       </c>
@@ -827,20 +837,23 @@
         <v>82</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
@@ -848,24 +861,27 @@
         <v>82</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="1"/>
       <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>89</v>
       </c>
@@ -873,24 +889,29 @@
         <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>89</v>
       </c>
@@ -898,24 +919,27 @@
         <v>82</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>89</v>
       </c>
@@ -923,26 +947,29 @@
         <v>82</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>102</v>
       </c>
       <c r="H6" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>89</v>
       </c>
@@ -950,26 +977,29 @@
         <v>82</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>89</v>
       </c>
@@ -977,26 +1007,29 @@
         <v>82</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>89</v>
       </c>
@@ -1004,26 +1037,29 @@
         <v>82</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>89</v>
       </c>
@@ -1031,26 +1067,29 @@
         <v>82</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>89</v>
       </c>
@@ -1058,20 +1097,23 @@
         <v>82</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>89</v>
       </c>
@@ -1079,850 +1121,967 @@
         <v>82</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="H23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="H24" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-    </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="E27" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J29" s="1"/>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J30" s="1"/>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J31" s="1"/>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J32" s="1"/>
+    </row>
+    <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J33" s="1"/>
+    </row>
+    <row r="34" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J34" s="1"/>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J35" s="1"/>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J36" s="1"/>
+    </row>
+    <row r="37" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J37" s="1"/>
+    </row>
+    <row r="38" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J38" s="1"/>
+    </row>
+    <row r="39" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-    </row>
-    <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J39" s="1"/>
+    </row>
+    <row r="40" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J40" s="1"/>
+    </row>
+    <row r="41" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J41" s="1"/>
+    </row>
+    <row r="42" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J42" s="1"/>
+    </row>
+    <row r="43" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J43" s="1"/>
+    </row>
+    <row r="44" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="E44" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="F44" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J44" s="1"/>
+    </row>
+    <row r="45" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
-    </row>
-    <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J45" s="1"/>
+    </row>
+    <row r="46" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="E46" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J46" s="1"/>
+    </row>
+    <row r="47" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="E47" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
-    </row>
-    <row r="48" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J47" s="1"/>
+    </row>
+    <row r="48" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="E48" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="F48" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="G48" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
-    </row>
-    <row r="49" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J48" s="1"/>
+    </row>
+    <row r="49" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="E49" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="F49" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="G49" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
-    </row>
-    <row r="50" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J49" s="1"/>
+    </row>
+    <row r="50" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="E50" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>